<commit_message>
Update prices from a 2026 search and confirm main links are live
- Re-priced the generic parts from a 3 Oct 2026 AliExpress search (power
  supply, Leonardo, belt, XT60 up; switches, Arca clamp/plate, SK8,
  wireless board, pulley down). Wheel about AUD 191, shifter AUD 65.50,
  pedals AUD 86.40, all three AUD 328.40 (AUD 196.10 with every
  trade-off).
- Opened every DAZ listing used as a main link to confirm it is live.
  The rim now uses DAZ's Europe link, the one confirmed live with his
  exact wheel.
- Local fallbacks: Bunnings 16 mm aluminium tube as the tube's backup,
  plus Jaycar part numbers for the Leonardo, XT60 and 608 bearings.
- Row heights now simulate word wrap, so long notes aren't cut off.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEYLvGWigrKvVwvVek2yBU
</commit_message>
<xml_diff>
--- a/parts-lists/DAZ-racing_pedal_set_budget_parts_list_AUD.xlsx
+++ b/parts-lists/DAZ-racing_pedal_set_budget_parts_list_AUD.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="159">
   <si>
     <t xml:space="preserve">DAZ Racing Load-Cell Pedal Set (throttle, brake, clutch) – budget parts list (AUD)</t>
   </si>
@@ -94,13 +94,13 @@
     <t xml:space="preserve">AliExpress search: 150 kg load cell</t>
   </si>
   <si>
-    <t xml:space="preserve">Link OK – page not auto-checked</t>
+    <t xml:space="preserve">Live (3 Oct 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">What makes the brake feel real. DAZ's brake pedal is designed for this load cell, so stick to his listing.</t>
   </si>
   <si>
-    <t xml:space="preserve">DAZ's link: €13.39 (May 2025) ≈ AUD 19.60 incl. GST.</t>
+    <t xml:space="preserve">DAZ's link: €13.39 (May 2025) ≈ AUD 19.60 incl. GST; 2026 search ≈ US$12.95 ≈ AUD 20.50.</t>
   </si>
   <si>
     <t xml:space="preserve">Arduino Leonardo R3 (ATmega32U4)</t>
@@ -115,10 +115,10 @@
     <t xml:space="preserve">Search – in-stock sellers</t>
   </si>
   <si>
-    <t xml:space="preserve">Any Leonardo R3 clone runs DAZ's pedal code. Need it today? Jaycar and Core Electronics sell compatible boards, but dearer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAZ's price column €5 ≈ AUD 7.30 incl. GST.</t>
+    <t xml:space="preserve">Any Leonardo R3 clone runs DAZ's pedal code. Need it today? Jaycar's Duinotech Leonardo (XC4430) is ≈ $35.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 search: Leonardo R3 clones ≈ US$7.31 (US store) ≈ AUD 11.60 incl. GST; DAZ's price column €5. Estimate AUD 10.</t>
   </si>
   <si>
     <t xml:space="preserve">HX711 load-cell amplifier</t>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">Keep the clutch: an H-pattern shifter needs one to feel right.</t>
   </si>
   <si>
-    <t xml:space="preserve">DAZ's price column €6 for six ≈ AUD 8.80.</t>
+    <t xml:space="preserve">2026 search: SK8 4-packs ≈ US$3.51 ≈ AUD 5.60 incl. GST (≈ AUD 1.40 each).</t>
   </si>
   <si>
     <t xml:space="preserve">Hall sensor module KY-035 (49E, analog)</t>
@@ -220,6 +220,9 @@
     <t xml:space="preserve">AliExpress search: 1.5 mm wire rope clip</t>
   </si>
   <si>
+    <t xml:space="preserve">DAZ's listing is a steel wire-rope clamp for 1.5–3 mm cable.</t>
+  </si>
+  <si>
     <t xml:space="preserve">DAZ's link: €3.41 (May 2025) ≈ AUD 5.</t>
   </si>
   <si>
@@ -373,7 +376,7 @@
     <t xml:space="preserve">An old bike's brake cables work, and bike shops often throw out offcuts – ask.</t>
   </si>
   <si>
-    <t xml:space="preserve">DAZ's link: €2.69 (May 2025) ≈ AUD 3.90.</t>
+    <t xml:space="preserve">DAZ's link: €2.69 (May 2025) ≈ AUD 3.90; 2026 search from US$0.87 per cable.</t>
   </si>
   <si>
     <t xml:space="preserve">Pedal base: bolt to your metal frame's pedal plate (or scrap plywood ≈10 mm)</t>
@@ -490,10 +493,10 @@
     <t xml:space="preserve">• Links: 'DAZ's link' = DAZ's own AliExpress (affiliate) listing – used where his printed parts need that exact part, and buying through it supports him. 'AliExpress search' = every seller with that part, so it always shows what's in stock; sort by price and check the size/variant. Choice-badge listings ship free over the threshold and arrive fastest.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Listing check (3 Oct 2026): every DAZ link was opened to confirm it still leads to a product page. AliExpress's bot check blocked some page loads, marked as not auto-checked – those links still work. Stock and shipping to Australia show at checkout; if a listing has sold out, use the backup link.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Price basis: DAZ's links carry the price from when he made them (mostly May 2025), quoted where available; other figures are typical 2026 AliExpress listings.</t>
+    <t xml:space="preserve">• Listing check (3 Oct 2026): all 76 of DAZ's links still lead to an AliExpress product, and every DAZ listing used as a main link was opened to confirm its product page is live. Rows marked 'not auto-checked' were blocked by AliExpress's bot check – the link itself works. Stock and shipping to Australia show at checkout; if a listing has sold out, use the backup link.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Price basis: DAZ's links carry the price from when he made them (mostly May 2025), quoted where available. '2026 search' figures are from AliExpress's US store on 3 Oct 2026; since 2025 US prices include import tariffs, so Australian prices are usually a little lower.</t>
   </si>
   <si>
     <t xml:space="preserve">• Based on DAZ Racing's load-cell pedal set parts list.</t>
@@ -1132,11 +1135,11 @@
       </c>
       <c r="E3" s="6" t="n">
         <f aca="false">E34</f>
-        <v>85.6</v>
+        <v>86.4</v>
       </c>
       <c r="F3" s="3" t="str">
         <f aca="false">IF($E$3&lt;=$B$3,"UNDER BUDGET – $"&amp;TEXT($B$3-$E$3,"0.00")&amp;" spare","OVER BUDGET by $"&amp;TEXT($E$3-$B$3,"0.00"))</f>
-        <v>UNDER BUDGET – $114.40 spare</v>
+        <v>UNDER BUDGET – $113.60 spare</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1232,7 +1235,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
         <v>26</v>
       </c>
@@ -1243,11 +1246,11 @@
         <v>1</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">C8*D8</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>27</v>
@@ -1358,11 +1361,11 @@
         <v>6</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">C11*D11</f>
-        <v>9.6</v>
+        <v>8.4</v>
       </c>
       <c r="F11" s="16" t="s">
         <v>27</v>
@@ -1464,7 +1467,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
         <v>53</v>
       </c>
@@ -1572,14 +1575,16 @@
       <c r="J16" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="K16" s="9"/>
+      <c r="K16" s="9" t="s">
+        <v>65</v>
+      </c>
       <c r="L16" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>63</v>
@@ -1604,26 +1609,26 @@
         <v>21</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J17" s="15" t="s">
         <v>23</v>
       </c>
       <c r="K17" s="9"/>
       <c r="L17" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B18" s="18"/>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
       <c r="E18" s="19" t="n">
         <f aca="false">SUM(E7:E17)</f>
-        <v>67.6</v>
+        <v>68.4</v>
       </c>
       <c r="F18" s="18"/>
       <c r="G18" s="18"/>
@@ -1635,7 +1640,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -1649,12 +1654,12 @@
       <c r="K20" s="8"/>
       <c r="L20" s="8"/>
     </row>
-    <row r="21" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>1</v>
@@ -1667,13 +1672,13 @@
         <v>1.5</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I21" s="14" t="s">
         <v>21</v>
@@ -1682,18 +1687,18 @@
         <v>29</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>1</v>
@@ -1706,13 +1711,13 @@
         <v>3</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I22" s="14" t="s">
         <v>21</v>
@@ -1721,18 +1726,18 @@
         <v>29</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>1</v>
@@ -1745,13 +1750,13 @@
         <v>1.5</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I23" s="20"/>
       <c r="J23" s="15" t="s">
@@ -1759,15 +1764,15 @@
       </c>
       <c r="K23" s="9"/>
       <c r="L23" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>1</v>
@@ -1780,13 +1785,13 @@
         <v>1</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I24" s="20"/>
       <c r="J24" s="15" t="s">
@@ -1794,12 +1799,12 @@
       </c>
       <c r="K24" s="9"/>
       <c r="L24" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>54</v>
@@ -1815,13 +1820,13 @@
         <v>1</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I25" s="14" t="s">
         <v>21</v>
@@ -1831,15 +1836,15 @@
       </c>
       <c r="K25" s="9"/>
       <c r="L25" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>1</v>
@@ -1852,13 +1857,13 @@
         <v>2.5</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>21</v>
@@ -1868,12 +1873,12 @@
       </c>
       <c r="K26" s="9"/>
       <c r="L26" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B27" s="9" t="s">
         <v>18</v>
@@ -1898,24 +1903,24 @@
         <v>21</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J27" s="15" t="s">
         <v>23</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>1</v>
@@ -1928,13 +1933,13 @@
         <v>1</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I28" s="14" t="s">
         <v>21</v>
@@ -1944,15 +1949,15 @@
       </c>
       <c r="K28" s="9"/>
       <c r="L28" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>1</v>
@@ -1965,13 +1970,13 @@
         <v>1</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I29" s="14" t="s">
         <v>21</v>
@@ -1981,12 +1986,12 @@
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B30" s="9" t="s">
         <v>54</v>
@@ -2002,13 +2007,13 @@
         <v>1</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I30" s="14" t="s">
         <v>21</v>
@@ -2018,12 +2023,12 @@
       </c>
       <c r="K30" s="9"/>
       <c r="L30" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>54</v>
@@ -2039,28 +2044,28 @@
         <v>2.5</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I31" s="20"/>
       <c r="J31" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B32" s="18"/>
       <c r="C32" s="18"/>
@@ -2079,14 +2084,14 @@
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B34" s="21"/>
       <c r="C34" s="21"/>
       <c r="D34" s="21"/>
       <c r="E34" s="22" t="n">
         <f aca="false">E18+E32</f>
-        <v>85.6</v>
+        <v>86.4</v>
       </c>
       <c r="F34" s="21"/>
       <c r="G34" s="21"/>
@@ -2098,7 +2103,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -2114,7 +2119,7 @@
     </row>
     <row r="37" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B37" s="9" t="s">
         <v>63</v>
@@ -2130,13 +2135,13 @@
         <v>4</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>21</v>
@@ -2145,15 +2150,15 @@
         <v>29</v>
       </c>
       <c r="K37" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L37" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>18</v>
@@ -2169,31 +2174,31 @@
         <v>12</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I38" s="20"/>
       <c r="J38" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="L38" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>1</v>
@@ -2206,27 +2211,27 @@
         <v>5</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H39" s="20"/>
       <c r="I39" s="20"/>
       <c r="J39" s="15"/>
       <c r="K39" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L39" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C40" s="10" t="n">
         <v>1</v>
@@ -2239,24 +2244,24 @@
         <v>22</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H40" s="20"/>
       <c r="I40" s="20"/>
       <c r="J40" s="15"/>
       <c r="K40" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L40" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>18</v>
@@ -2272,24 +2277,24 @@
         <v>3</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H41" s="20"/>
       <c r="I41" s="20"/>
       <c r="J41" s="15"/>
       <c r="K41" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L41" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B42" s="18"/>
       <c r="C42" s="18"/>
@@ -2308,16 +2313,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E43" s="6" t="n">
         <f aca="false">E34+E42</f>
-        <v>131.6</v>
+        <v>132.4</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -2333,7 +2338,7 @@
     </row>
     <row r="46" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>63</v>
@@ -2349,7 +2354,7 @@
         <v>1.5</v>
       </c>
       <c r="F46" s="24" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>20</v>
@@ -2358,21 +2363,21 @@
         <v>21</v>
       </c>
       <c r="I46" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J46" s="15" t="s">
         <v>23</v>
       </c>
       <c r="K46" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L46" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
@@ -2391,16 +2396,16 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E48" s="6" t="n">
         <f aca="false">E34+E47</f>
-        <v>87.1</v>
+        <v>87.9</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -2416,7 +2421,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="25" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
@@ -2432,7 +2437,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="25" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B52" s="25"/>
       <c r="C52" s="25"/>
@@ -2448,7 +2453,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
@@ -2464,7 +2469,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="26" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B55" s="26"/>
       <c r="C55" s="26"/>
@@ -2480,7 +2485,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="26" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B56" s="26"/>
       <c r="C56" s="26"/>
@@ -2496,7 +2501,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B57" s="26"/>
       <c r="C57" s="26"/>
@@ -2512,7 +2517,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B58" s="26"/>
       <c r="C58" s="26"/>
@@ -2528,7 +2533,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B59" s="26"/>
       <c r="C59" s="26"/>
@@ -2544,7 +2549,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B60" s="26"/>
       <c r="C60" s="26"/>

</xml_diff>